<commit_message>
Deploy codeforIATI/codelists to github.com/codeforIATI/codelists.git:gh-pages
</commit_message>
<xml_diff>
--- a/api/clv1/codelist/CRSChannelCode.xlsx
+++ b/api/clv1/codelist/CRSChannelCode.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="721">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1177" uniqueCount="766">
   <si>
     <t>code</t>
   </si>
@@ -331,6 +331,12 @@
     <t>World Vision</t>
   </si>
   <si>
+    <t>21064</t>
+  </si>
+  <si>
+    <t>Clinton Health Access Initiative, Inc.</t>
+  </si>
+  <si>
     <t>22000</t>
   </si>
   <si>
@@ -535,6 +541,12 @@
     <t>Cities Alliance</t>
   </si>
   <si>
+    <t>31006</t>
+  </si>
+  <si>
+    <t>Coalition for Epidemic Preparedness Innovations</t>
+  </si>
+  <si>
     <t>30016</t>
   </si>
   <si>
@@ -811,6 +823,12 @@
     <t>Joint United Nations Programme on HIV/AIDS</t>
   </si>
   <si>
+    <t>41320</t>
+  </si>
+  <si>
+    <t>Technology Bank for Least Developed Countries</t>
+  </si>
+  <si>
     <t>41305</t>
   </si>
   <si>
@@ -844,7 +862,7 @@
     <t>41310</t>
   </si>
   <si>
-    <t>United Nations Department of Peacekeeping Operations [only MINURSO, MINUSCA, MINUSMA, MINUSTAH, MONUSCO, UNAMID, UNIFIL, UNISFA, UNMIK, UNMIL, UNMISS, UNOCI]. Report contributions mission by mission in CRS++.</t>
+    <t>United Nations Department of Peacekeeping Operations [only MINURSO, MINUSCA, MINUSMA, MINUJUSTH, MONUSCO, UNAMID, UNIFIL, UNISFA, UNMIK, UNMIL, UNMISS, UNOCI]. Report contributions mission by mission in CRS++.</t>
   </si>
   <si>
     <t>41148</t>
@@ -1246,7 +1264,7 @@
     <t>46008</t>
   </si>
   <si>
-    <t>Andean Development Corporation</t>
+    <t>Development Bank of Latin America</t>
   </si>
   <si>
     <t>46004</t>
@@ -1687,6 +1705,30 @@
     <t>International Organisation for Migration</t>
   </si>
   <si>
+    <t>41149</t>
+  </si>
+  <si>
+    <t>United Nations Development Coordination Office</t>
+  </si>
+  <si>
+    <t>41150</t>
+  </si>
+  <si>
+    <t>United Nations Institute for Disarmament Research</t>
+  </si>
+  <si>
+    <t>46027</t>
+  </si>
+  <si>
+    <t>Financial Fund for the Development of the River Plate Basin</t>
+  </si>
+  <si>
+    <t>47400</t>
+  </si>
+  <si>
+    <t>European Space Agency (ESA) programme “Space in support of International Development Aid”</t>
+  </si>
+  <si>
     <t>47046</t>
   </si>
   <si>
@@ -1915,6 +1957,24 @@
     <t>International Renewable Energy Agency</t>
   </si>
   <si>
+    <t>47146</t>
+  </si>
+  <si>
+    <t>International Investment Bank (IIB)</t>
+  </si>
+  <si>
+    <t>47147</t>
+  </si>
+  <si>
+    <t>International Finance Facility for Education</t>
+  </si>
+  <si>
+    <t>47148</t>
+  </si>
+  <si>
+    <t>World Organisation for Animal Health</t>
+  </si>
+  <si>
     <t>50000</t>
   </si>
   <si>
@@ -2113,7 +2173,7 @@
     <t>61001</t>
   </si>
   <si>
-    <t>Private bank in provider country</t>
+    <t>Banks (deposit taking corporations)</t>
   </si>
   <si>
     <t>61002</t>
@@ -2125,13 +2185,49 @@
     <t>61003</t>
   </si>
   <si>
-    <t>Private investor in provider country</t>
+    <t>Investment funds and other collective investment institutions</t>
   </si>
   <si>
     <t>61004</t>
   </si>
   <si>
-    <t>Other non-bank entity in provider country</t>
+    <t>Holding companies, trusts and Special Purpose Vehicles</t>
+  </si>
+  <si>
+    <t>61005</t>
+  </si>
+  <si>
+    <t>Insurance Corporations</t>
+  </si>
+  <si>
+    <t>61006</t>
+  </si>
+  <si>
+    <t>Pension Funds</t>
+  </si>
+  <si>
+    <t>61007</t>
+  </si>
+  <si>
+    <t>Other financial corporations</t>
+  </si>
+  <si>
+    <t>61008</t>
+  </si>
+  <si>
+    <t>Exporters</t>
+  </si>
+  <si>
+    <t>61009</t>
+  </si>
+  <si>
+    <t>Other non-financial corporations</t>
+  </si>
+  <si>
+    <t>61010</t>
+  </si>
+  <si>
+    <t>Retail investors</t>
   </si>
   <si>
     <t>62000</t>
@@ -2143,19 +2239,40 @@
     <t>62001</t>
   </si>
   <si>
-    <t>Private bank in recipient country</t>
+    <t>Banks (deposit taking corporations except Micro Finance Institutions)</t>
   </si>
   <si>
     <t>62002</t>
   </si>
   <si>
-    <t>Joint-venture in recipient country</t>
+    <t>Micro Finance Institutions (deposit and non-deposit)</t>
   </si>
   <si>
     <t>62003</t>
   </si>
   <si>
-    <t>Other non-bank in recipient country</t>
+    <t>62004</t>
+  </si>
+  <si>
+    <t>62005</t>
+  </si>
+  <si>
+    <t>62006</t>
+  </si>
+  <si>
+    <t>62007</t>
+  </si>
+  <si>
+    <t>62008</t>
+  </si>
+  <si>
+    <t>Importers/Exporters</t>
+  </si>
+  <si>
+    <t>62009</t>
+  </si>
+  <si>
+    <t>62010</t>
   </si>
   <si>
     <t>63000</t>
@@ -2167,13 +2284,31 @@
     <t>63001</t>
   </si>
   <si>
-    <t>Private bank in third country</t>
-  </si>
-  <si>
     <t>63002</t>
   </si>
   <si>
-    <t>Private non-bank in third country</t>
+    <t>63003</t>
+  </si>
+  <si>
+    <t>63004</t>
+  </si>
+  <si>
+    <t>63005</t>
+  </si>
+  <si>
+    <t>63006</t>
+  </si>
+  <si>
+    <t>63007</t>
+  </si>
+  <si>
+    <t>63008</t>
+  </si>
+  <si>
+    <t>63009</t>
+  </si>
+  <si>
+    <t>63010</t>
   </si>
   <si>
     <t>90000</t>
@@ -2508,7 +2643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G360"/>
+  <dimension ref="A1:G391"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -6323,7 +6458,7 @@
         <v>693</v>
       </c>
       <c r="B346" t="s">
-        <v>634</v>
+        <v>694</v>
       </c>
       <c r="D346" t="s">
         <v>9</v>
@@ -6331,10 +6466,10 @@
     </row>
     <row r="347" spans="1:4">
       <c r="A347" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B347" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="D347" t="s">
         <v>9</v>
@@ -6342,10 +6477,10 @@
     </row>
     <row r="348" spans="1:4">
       <c r="A348" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B348" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="D348" t="s">
         <v>9</v>
@@ -6353,10 +6488,10 @@
     </row>
     <row r="349" spans="1:4">
       <c r="A349" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B349" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="D349" t="s">
         <v>9</v>
@@ -6364,10 +6499,10 @@
     </row>
     <row r="350" spans="1:4">
       <c r="A350" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B350" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="D350" t="s">
         <v>9</v>
@@ -6375,10 +6510,10 @@
     </row>
     <row r="351" spans="1:4">
       <c r="A351" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B351" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="D351" t="s">
         <v>9</v>
@@ -6386,10 +6521,10 @@
     </row>
     <row r="352" spans="1:4">
       <c r="A352" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B352" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="D352" t="s">
         <v>9</v>
@@ -6397,10 +6532,10 @@
     </row>
     <row r="353" spans="1:4">
       <c r="A353" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B353" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="D353" t="s">
         <v>9</v>
@@ -6408,10 +6543,10 @@
     </row>
     <row r="354" spans="1:4">
       <c r="A354" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B354" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="D354" t="s">
         <v>9</v>
@@ -6419,10 +6554,10 @@
     </row>
     <row r="355" spans="1:4">
       <c r="A355" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B355" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="D355" t="s">
         <v>9</v>
@@ -6430,10 +6565,10 @@
     </row>
     <row r="356" spans="1:4">
       <c r="A356" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B356" t="s">
-        <v>713</v>
+        <v>654</v>
       </c>
       <c r="D356" t="s">
         <v>9</v>
@@ -6477,9 +6612,350 @@
         <v>720</v>
       </c>
       <c r="B360" t="s">
-        <v>634</v>
+        <v>721</v>
       </c>
       <c r="D360" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="361" spans="1:4">
+      <c r="A361" t="s">
+        <v>722</v>
+      </c>
+      <c r="B361" t="s">
+        <v>723</v>
+      </c>
+      <c r="D361" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="362" spans="1:4">
+      <c r="A362" t="s">
+        <v>724</v>
+      </c>
+      <c r="B362" t="s">
+        <v>725</v>
+      </c>
+      <c r="D362" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="363" spans="1:4">
+      <c r="A363" t="s">
+        <v>726</v>
+      </c>
+      <c r="B363" t="s">
+        <v>727</v>
+      </c>
+      <c r="D363" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="364" spans="1:4">
+      <c r="A364" t="s">
+        <v>728</v>
+      </c>
+      <c r="B364" t="s">
+        <v>729</v>
+      </c>
+      <c r="D364" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="365" spans="1:4">
+      <c r="A365" t="s">
+        <v>730</v>
+      </c>
+      <c r="B365" t="s">
+        <v>731</v>
+      </c>
+      <c r="D365" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="366" spans="1:4">
+      <c r="A366" t="s">
+        <v>732</v>
+      </c>
+      <c r="B366" t="s">
+        <v>733</v>
+      </c>
+      <c r="D366" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="367" spans="1:4">
+      <c r="A367" t="s">
+        <v>734</v>
+      </c>
+      <c r="B367" t="s">
+        <v>735</v>
+      </c>
+      <c r="D367" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="368" spans="1:4">
+      <c r="A368" t="s">
+        <v>736</v>
+      </c>
+      <c r="B368" t="s">
+        <v>737</v>
+      </c>
+      <c r="D368" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="369" spans="1:4">
+      <c r="A369" t="s">
+        <v>738</v>
+      </c>
+      <c r="B369" t="s">
+        <v>739</v>
+      </c>
+      <c r="D369" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="370" spans="1:4">
+      <c r="A370" t="s">
+        <v>740</v>
+      </c>
+      <c r="B370" t="s">
+        <v>741</v>
+      </c>
+      <c r="D370" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="371" spans="1:4">
+      <c r="A371" t="s">
+        <v>742</v>
+      </c>
+      <c r="B371" t="s">
+        <v>743</v>
+      </c>
+      <c r="D371" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="372" spans="1:4">
+      <c r="A372" t="s">
+        <v>744</v>
+      </c>
+      <c r="B372" t="s">
+        <v>723</v>
+      </c>
+      <c r="D372" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="373" spans="1:4">
+      <c r="A373" t="s">
+        <v>745</v>
+      </c>
+      <c r="B373" t="s">
+        <v>725</v>
+      </c>
+      <c r="D373" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="374" spans="1:4">
+      <c r="A374" t="s">
+        <v>746</v>
+      </c>
+      <c r="B374" t="s">
+        <v>727</v>
+      </c>
+      <c r="D374" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="375" spans="1:4">
+      <c r="A375" t="s">
+        <v>747</v>
+      </c>
+      <c r="B375" t="s">
+        <v>729</v>
+      </c>
+      <c r="D375" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="376" spans="1:4">
+      <c r="A376" t="s">
+        <v>748</v>
+      </c>
+      <c r="B376" t="s">
+        <v>731</v>
+      </c>
+      <c r="D376" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="377" spans="1:4">
+      <c r="A377" t="s">
+        <v>749</v>
+      </c>
+      <c r="B377" t="s">
+        <v>750</v>
+      </c>
+      <c r="D377" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="378" spans="1:4">
+      <c r="A378" t="s">
+        <v>751</v>
+      </c>
+      <c r="B378" t="s">
+        <v>735</v>
+      </c>
+      <c r="D378" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="379" spans="1:4">
+      <c r="A379" t="s">
+        <v>752</v>
+      </c>
+      <c r="B379" t="s">
+        <v>737</v>
+      </c>
+      <c r="D379" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="380" spans="1:4">
+      <c r="A380" t="s">
+        <v>753</v>
+      </c>
+      <c r="B380" t="s">
+        <v>754</v>
+      </c>
+      <c r="D380" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="381" spans="1:4">
+      <c r="A381" t="s">
+        <v>755</v>
+      </c>
+      <c r="B381" t="s">
+        <v>741</v>
+      </c>
+      <c r="D381" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="382" spans="1:4">
+      <c r="A382" t="s">
+        <v>756</v>
+      </c>
+      <c r="B382" t="s">
+        <v>743</v>
+      </c>
+      <c r="D382" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="383" spans="1:4">
+      <c r="A383" t="s">
+        <v>757</v>
+      </c>
+      <c r="B383" t="s">
+        <v>723</v>
+      </c>
+      <c r="D383" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="384" spans="1:4">
+      <c r="A384" t="s">
+        <v>758</v>
+      </c>
+      <c r="B384" t="s">
+        <v>725</v>
+      </c>
+      <c r="D384" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="385" spans="1:4">
+      <c r="A385" t="s">
+        <v>759</v>
+      </c>
+      <c r="B385" t="s">
+        <v>727</v>
+      </c>
+      <c r="D385" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="386" spans="1:4">
+      <c r="A386" t="s">
+        <v>760</v>
+      </c>
+      <c r="B386" t="s">
+        <v>729</v>
+      </c>
+      <c r="D386" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="387" spans="1:4">
+      <c r="A387" t="s">
+        <v>761</v>
+      </c>
+      <c r="B387" t="s">
+        <v>731</v>
+      </c>
+      <c r="D387" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="388" spans="1:4">
+      <c r="A388" t="s">
+        <v>762</v>
+      </c>
+      <c r="B388" t="s">
+        <v>733</v>
+      </c>
+      <c r="D388" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="389" spans="1:4">
+      <c r="A389" t="s">
+        <v>763</v>
+      </c>
+      <c r="B389" t="s">
+        <v>735</v>
+      </c>
+      <c r="D389" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="390" spans="1:4">
+      <c r="A390" t="s">
+        <v>764</v>
+      </c>
+      <c r="B390" t="s">
+        <v>737</v>
+      </c>
+      <c r="D390" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="391" spans="1:4">
+      <c r="A391" t="s">
+        <v>765</v>
+      </c>
+      <c r="B391" t="s">
+        <v>654</v>
+      </c>
+      <c r="D391" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>